<commit_message>
week 8 assessment shared
</commit_message>
<xml_diff>
--- a/Exercises/CU-.NET-Batch4-Assignments-Repositories.xlsx
+++ b/Exercises/CU-.NET-Batch4-Assignments-Repositories.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Trainings\2025-Freelance\2026 01 DotNet CHD Capgemini\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Trainings\2025-Freelance\2026 01 DotNet CHD Capgemini\CU-DotNet-Jan26-B4\Exercises\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FFC7E408-1207-449C-9BF8-52D1EB2CCC26}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0300E9E2-1477-4F86-A439-913A24737CB7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{C99DFE55-A9F3-4CE7-8732-71313EE2B406}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="43">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="44">
   <si>
     <t>SNO</t>
   </si>
@@ -163,6 +163,9 @@
   </si>
   <si>
     <t>Day10-01 Methods Orders.docx</t>
+  </si>
+  <si>
+    <t>Day46-Week8 Assessment NUnit.docx</t>
   </si>
 </sst>
 </file>
@@ -867,6 +870,9 @@
       <c r="A40" s="1">
         <v>39</v>
       </c>
+      <c r="B40" t="s">
+        <v>43</v>
+      </c>
     </row>
     <row r="41" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A41" s="1">

</xml_diff>